<commit_message>
Increased network size, allowed more reactions to be adde, increase risk to 99 percent, increased the minimum entropy weight. The run seems promising. Added saved models to gitignore.
</commit_message>
<xml_diff>
--- a/Testing_Feedback/Discover_Molecular_Integrators.xlsx
+++ b/Testing_Feedback/Discover_Molecular_Integrators.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,7 +424,42 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2025-05-14 20:52:16</t>
+          <t>2025-05-16 13:46:50</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>2025-05-16 14:22:38</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>2025-05-16 15:04:55</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>2025-05-16 15:25:36</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>2025-05-16 16:25:59</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>2025-05-17 11:54:25</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>2025-05-17 13:09:27</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>2025-05-17 14:42:30</t>
         </is>
       </c>
     </row>
@@ -436,7 +471,42 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.comet.com/maurice-filo/molecular-integrators/2e4d7905602e44a2845a562e68b0c6cf</t>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/50336799a8e64cda9b072c848a054cd6</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/8cd58232b88148c1b833ab5c8c4ab676</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/cf3e4262a9384f4cbe47e620d930816a</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/5885b3f22de74ab78df9adb046aa8c47</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/8e8f71c6cf424bcabfc95ba7fd183d1f</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/46d1628ad23a43cc8b1f3bab2e365bb4</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/4cbf7319c2e2484f8262574ffd5e4f2c</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/maurice-filo/molecular-integrators/bbc345cfb544454ba9960aa8c4e6d17f</t>
         </is>
       </c>
     </row>
@@ -447,7 +517,28 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -457,7 +548,28 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1280</v>
+        <v>3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -467,7 +579,28 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>200</v>
+        <v>2</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -476,8 +609,29 @@
           <t>Number of Samples</t>
         </is>
       </c>
-      <c r="B6" t="b">
-        <v>0</v>
+      <c r="B6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1280</v>
       </c>
     </row>
     <row r="7">
@@ -487,7 +641,28 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1e-05</v>
+        <v>200</v>
+      </c>
+      <c r="C7" t="n">
+        <v>200</v>
+      </c>
+      <c r="D7" t="n">
+        <v>200</v>
+      </c>
+      <c r="E7" t="n">
+        <v>200</v>
+      </c>
+      <c r="F7" t="n">
+        <v>200</v>
+      </c>
+      <c r="G7" t="n">
+        <v>200</v>
+      </c>
+      <c r="H7" t="n">
+        <v>200</v>
+      </c>
+      <c r="I7" t="n">
+        <v>200</v>
       </c>
     </row>
     <row r="8">
@@ -496,8 +671,29 @@
           <t>Allow Input Influence</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>100</v>
+      <c r="B8" t="b">
+        <v>0</v>
+      </c>
+      <c r="C8" t="b">
+        <v>0</v>
+      </c>
+      <c r="D8" t="b">
+        <v>0</v>
+      </c>
+      <c r="E8" t="b">
+        <v>0</v>
+      </c>
+      <c r="F8" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8" t="b">
+        <v>0</v>
+      </c>
+      <c r="H8" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -507,7 +703,28 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.75</v>
+        <v>1e-06</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1e-06</v>
       </c>
     </row>
     <row r="10">
@@ -517,7 +734,28 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5</v>
+        <v>100</v>
+      </c>
+      <c r="C10" t="n">
+        <v>100</v>
+      </c>
+      <c r="D10" t="n">
+        <v>100</v>
+      </c>
+      <c r="E10" t="n">
+        <v>100</v>
+      </c>
+      <c r="F10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G10" t="n">
+        <v>100</v>
+      </c>
+      <c r="H10" t="n">
+        <v>100</v>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="11">
@@ -527,7 +765,28 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>0.75</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.75</v>
       </c>
     </row>
     <row r="12">
@@ -537,7 +796,28 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="C12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H12" t="n">
+        <v>5</v>
+      </c>
+      <c r="I12" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -547,7 +827,28 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="C13" t="n">
+        <v>10</v>
+      </c>
+      <c r="D13" t="n">
+        <v>10</v>
+      </c>
+      <c r="E13" t="n">
+        <v>10</v>
+      </c>
+      <c r="F13" t="n">
+        <v>10</v>
+      </c>
+      <c r="G13" t="n">
+        <v>10</v>
+      </c>
+      <c r="H13" t="n">
+        <v>10</v>
+      </c>
+      <c r="I13" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="14">
@@ -557,7 +858,28 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.99</v>
       </c>
     </row>
     <row r="15">
@@ -567,7 +889,28 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>20</v>
+        <v>0</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -577,7 +920,28 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1000</v>
+        <v>1</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -587,7 +951,28 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5</v>
+        <v>20</v>
+      </c>
+      <c r="C17" t="n">
+        <v>20</v>
+      </c>
+      <c r="D17" t="n">
+        <v>20</v>
+      </c>
+      <c r="E17" t="n">
+        <v>20</v>
+      </c>
+      <c r="F17" t="n">
+        <v>20</v>
+      </c>
+      <c r="G17" t="n">
+        <v>20</v>
+      </c>
+      <c r="H17" t="n">
+        <v>20</v>
+      </c>
+      <c r="I17" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="18">
@@ -597,7 +982,28 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>5</v>
+        <v>1000</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I18" t="n">
+        <v>3000</v>
       </c>
     </row>
     <row r="19">
@@ -607,7 +1013,28 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1024</v>
+        <v>10</v>
+      </c>
+      <c r="C19" t="n">
+        <v>10</v>
+      </c>
+      <c r="D19" t="n">
+        <v>10</v>
+      </c>
+      <c r="E19" t="n">
+        <v>10</v>
+      </c>
+      <c r="F19" t="n">
+        <v>10</v>
+      </c>
+      <c r="G19" t="n">
+        <v>10</v>
+      </c>
+      <c r="H19" t="n">
+        <v>10</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -617,7 +1044,28 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>128</v>
+        <v>5</v>
+      </c>
+      <c r="C20" t="n">
+        <v>5</v>
+      </c>
+      <c r="D20" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" t="n">
+        <v>5</v>
+      </c>
+      <c r="F20" t="n">
+        <v>5</v>
+      </c>
+      <c r="G20" t="n">
+        <v>5</v>
+      </c>
+      <c r="H20" t="n">
+        <v>5</v>
+      </c>
+      <c r="I20" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="21">
@@ -626,12 +1074,60 @@
           <t>Neural Network Width</t>
         </is>
       </c>
+      <c r="B21" t="n">
+        <v>1024</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1024</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1024</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1024</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1024</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1024</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1024</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1024</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
           <t>Number of CPUs</t>
         </is>
+      </c>
+      <c r="B22" t="n">
+        <v>128</v>
+      </c>
+      <c r="C22" t="n">
+        <v>128</v>
+      </c>
+      <c r="D22" t="n">
+        <v>128</v>
+      </c>
+      <c r="E22" t="n">
+        <v>128</v>
+      </c>
+      <c r="F22" t="n">
+        <v>128</v>
+      </c>
+      <c r="G22" t="n">
+        <v>128</v>
+      </c>
+      <c r="H22" t="n">
+        <v>128</v>
+      </c>
+      <c r="I22" t="n">
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>